<commit_message>
:white_circle: Dev v5.10: Correcciones de imágenes Marcelo Perez
</commit_message>
<xml_diff>
--- a/02_Codigo/03_HybridTugboat/01_codes/01_Pnom015/Comparation_015.xlsx
+++ b/02_Codigo/03_HybridTugboat/01_codes/01_Pnom015/Comparation_015.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\03_HybridTugboat\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B0282D8-F777-435A-BF45-3EF4A2AC7E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1FDBD3-88C0-4BDD-A241-54F2F6D2AA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{CC8E70EA-9981-4FE1-9A98-EC6DB5F1210E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{CC8E70EA-9981-4FE1-9A98-EC6DB5F1210E}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Maneuver" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="14">
   <si>
     <t>Pot_acc [kW]</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Hybrid Tug 15% Pnom</t>
+  </si>
+  <si>
+    <t>Batt</t>
   </si>
 </sst>
 </file>
@@ -130,7 +133,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -139,6 +142,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,6 +519,7 @@
       <c r="H3" t="s">
         <v>2</v>
       </c>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
@@ -534,6 +540,7 @@
       <c r="H4" s="1">
         <v>1.2733531401</v>
       </c>
+      <c r="K4" s="1"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
@@ -582,11 +589,26 @@
       <c r="D7" s="1">
         <v>14.325076506750001</v>
       </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
       <c r="G7" s="1">
-        <v>2405.4780240240243</v>
+        <f>C7-SUM(G4:G6)</f>
+        <v>2960.0658198198198</v>
       </c>
       <c r="H7" s="1">
-        <v>6.4222113791849997</v>
+        <f>D7-SUM(H4:H6)</f>
+        <v>7.9028651275650015</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G8" s="6">
+        <f>SUM(G4:G7)</f>
+        <v>5365.5438438438441</v>
+      </c>
+      <c r="H8" s="6">
+        <f>SUM(H4:H7)</f>
+        <v>14.325076506750001</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -651,12 +673,12 @@
         <v>3</v>
       </c>
       <c r="G11" s="2">
-        <f>G4/$G$7</f>
-        <v>0.19827331504955736</v>
+        <f>G4/$G$8</f>
+        <v>8.8889796818885661E-2</v>
       </c>
       <c r="H11" s="2">
-        <f>H4/$H$7</f>
-        <v>0.19827331504955739</v>
+        <f>H4/$H$8</f>
+        <v>8.8889796818885661E-2</v>
       </c>
       <c r="J11" t="s">
         <v>3</v>
@@ -686,12 +708,12 @@
         <v>4</v>
       </c>
       <c r="G12" s="2">
-        <f t="shared" ref="G12:G13" si="2">G5/$G$7</f>
-        <v>0.4240792845377544</v>
+        <f>G5/$G$8</f>
+        <v>0.1901230199749139</v>
       </c>
       <c r="H12" s="2">
-        <f t="shared" ref="H12:H13" si="3">H5/$H$7</f>
-        <v>0.42407928453775445</v>
+        <f>H5/$H$8</f>
+        <v>0.19012301997491388</v>
       </c>
       <c r="J12" t="s">
         <v>4</v>
@@ -701,7 +723,7 @@
         <v>0.1901230199749139</v>
       </c>
       <c r="L12" s="2">
-        <f t="shared" ref="L12:L13" si="4">H5/$D$7</f>
+        <f t="shared" ref="L12:L13" si="2">H5/$D$7</f>
         <v>0.19012301997491388</v>
       </c>
     </row>
@@ -721,22 +743,22 @@
         <v>7</v>
       </c>
       <c r="G13" s="2">
-        <f t="shared" si="2"/>
-        <v>0.37764740041268813</v>
+        <f>G6/$G$8</f>
+        <v>0.16930670011480775</v>
       </c>
       <c r="H13" s="2">
-        <f t="shared" si="3"/>
-        <v>0.37764740041268818</v>
+        <f>H6/$H$8</f>
+        <v>0.16930670011480775</v>
       </c>
       <c r="J13" t="s">
         <v>7</v>
       </c>
       <c r="K13" s="2">
-        <f t="shared" ref="K13" si="5">G6/$C$7</f>
+        <f t="shared" ref="K13" si="3">G6/$C$7</f>
         <v>0.16930670011480775</v>
       </c>
       <c r="L13" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0.16930670011480775</v>
       </c>
     </row>
@@ -749,13 +771,16 @@
         <f>SUM(D11:D13)</f>
         <v>0.99999999999999989</v>
       </c>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
       <c r="G14" s="2">
-        <f>SUM(G11:G13)</f>
-        <v>1</v>
+        <f>G7/$G$8</f>
+        <v>0.55168048309139261</v>
       </c>
       <c r="H14" s="2">
-        <f>SUM(H11:H13)</f>
-        <v>1</v>
+        <f>H7/$H$8</f>
+        <v>0.55168048309139273</v>
       </c>
       <c r="K14" s="2">
         <f>SUM(K11:K13)</f>
@@ -766,13 +791,23 @@
         <v>0.44831951690860727</v>
       </c>
     </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G15" s="7">
+        <f>SUM(G11:G14)</f>
+        <v>1</v>
+      </c>
+      <c r="H15" s="7">
+        <f>SUM(H11:H14)</f>
+        <v>1</v>
+      </c>
+    </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="J16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="K16" s="4">
-        <f>1-G7/C7</f>
-        <v>0.55168048309139261</v>
+        <f>1-G8/C7</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
:green_circle: Dev v6.0: Tesis v1.0
</commit_message>
<xml_diff>
--- a/02_Codigo/03_HybridTugboat/01_codes/01_Pnom015/Comparation_015.xlsx
+++ b/02_Codigo/03_HybridTugboat/01_codes/01_Pnom015/Comparation_015.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\03_HybridTugboat\01_codes\01_Pnom015\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\03_HybridTugboat\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1FDBD3-88C0-4BDD-A241-54F2F6D2AA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD417CA-D16C-4C17-912A-CDAC20A26297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{CC8E70EA-9981-4FE1-9A98-EC6DB5F1210E}"/>
+    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{CC8E70EA-9981-4FE1-9A98-EC6DB5F1210E}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Maneuver" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="15">
   <si>
     <t>Pot_acc [kW]</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Batt</t>
+  </si>
+  <si>
+    <t>Total Consumption</t>
   </si>
 </sst>
 </file>
@@ -139,11 +142,11 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,28 +482,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F86E1CB-682A-45B9-8296-40FE06F59BBE}">
-  <dimension ref="B2:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:L25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -521,7 +524,7 @@
       </c>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -540,9 +543,15 @@
       <c r="H4" s="1">
         <v>1.2733531401</v>
       </c>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="1">
+        <f>SUM(G4:G6)</f>
+        <v>2405.4780240240243</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -562,7 +571,7 @@
         <v>2.7235268068349998</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -582,7 +591,7 @@
         <v>2.4253314322500001</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C7" s="1">
         <v>5365.5438438438441</v>
       </c>
@@ -601,222 +610,279 @@
         <v>7.9028651275650015</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="G8" s="6">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="G8" s="5">
         <f>SUM(G4:G7)</f>
         <v>5365.5438438438441</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <f>SUM(H4:H7)</f>
         <v>14.325076506750001</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="F9" s="5" t="s">
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="F10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="J9" s="5" t="s">
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="J10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
         <v>0</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>8</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F11" t="s">
         <v>0</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G11" t="s">
         <v>8</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H11" t="s">
         <v>9</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J11" t="s">
         <v>0</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K11" t="s">
         <v>8</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C12" s="2">
         <f>C4/$C$7</f>
         <v>0.39079576886462902</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D12" s="2">
         <f>D4/$D$7</f>
         <v>0.39079576886462902</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F12" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G12" s="2">
         <f>G4/$G$8</f>
         <v>8.8889796818885661E-2</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H12" s="2">
         <f>H4/$H$8</f>
         <v>8.8889796818885661E-2</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J12" t="s">
         <v>3</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K12" s="2">
         <f>G4/$C$7</f>
         <v>8.8889796818885661E-2</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L12" s="2">
         <f>H4/$D$7</f>
         <v>8.8889796818885661E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="2">
-        <f t="shared" ref="C12:C13" si="0">C5/$C$7</f>
+      <c r="C13" s="2">
+        <f>C5/$C$7</f>
         <v>0.43989753102056328</v>
       </c>
-      <c r="D12" s="2">
-        <f t="shared" ref="D12:D13" si="1">D5/$D$7</f>
+      <c r="D13" s="2">
+        <f>D5/$D$7</f>
         <v>0.43989753102056317</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G13" s="2">
         <f>G5/$G$8</f>
         <v>0.1901230199749139</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H13" s="2">
         <f>H5/$H$8</f>
         <v>0.19012301997491388</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J13" t="s">
         <v>4</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K13" s="2">
         <f>G5/$C$7</f>
         <v>0.1901230199749139</v>
       </c>
-      <c r="L12" s="2">
-        <f t="shared" ref="L12:L13" si="2">H5/$D$7</f>
+      <c r="L13" s="2">
+        <f>H5/$D$7</f>
         <v>0.19012301997491388</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="2">
-        <f t="shared" si="0"/>
+      <c r="C14" s="2">
+        <f>C6/$C$7</f>
         <v>0.16930670011480775</v>
       </c>
-      <c r="D13" s="2">
-        <f t="shared" si="1"/>
+      <c r="D14" s="2">
+        <f>D6/$D$7</f>
         <v>0.16930670011480775</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F14" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G14" s="2">
         <f>G6/$G$8</f>
         <v>0.16930670011480775</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H14" s="2">
         <f>H6/$H$8</f>
         <v>0.16930670011480775</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J14" t="s">
         <v>7</v>
       </c>
-      <c r="K13" s="2">
-        <f t="shared" ref="K13" si="3">G6/$C$7</f>
+      <c r="K14" s="2">
+        <f>G6/$C$7</f>
         <v>0.16930670011480775</v>
       </c>
-      <c r="L13" s="2">
-        <f t="shared" si="2"/>
+      <c r="L14" s="2">
+        <f>H6/$D$7</f>
         <v>0.16930670011480775</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C14" s="2">
-        <f>SUM(C11:C13)</f>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C15" s="2">
+        <f>SUM(C12:C14)</f>
         <v>1</v>
       </c>
-      <c r="D14" s="2">
-        <f>SUM(D11:D13)</f>
+      <c r="D15" s="2">
+        <f>SUM(D12:D14)</f>
         <v>0.99999999999999989</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F15" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G15" s="2">
         <f>G7/$G$8</f>
         <v>0.55168048309139261</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H15" s="2">
         <f>H7/$H$8</f>
         <v>0.55168048309139273</v>
       </c>
-      <c r="K14" s="2">
-        <f>SUM(K11:K13)</f>
+      <c r="K15" s="2">
+        <f>SUM(K12:K14)</f>
         <v>0.44831951690860733</v>
       </c>
-      <c r="L14" s="2">
-        <f>SUM(L11:L13)</f>
+      <c r="L15" s="2">
+        <f>SUM(L12:L14)</f>
         <v>0.44831951690860727</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="G15" s="7">
-        <f>SUM(G11:G14)</f>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="G16" s="6">
+        <f>SUM(G12:G15)</f>
         <v>1</v>
       </c>
-      <c r="H15" s="7">
-        <f>SUM(H11:H14)</f>
+      <c r="H16" s="6">
+        <f>SUM(H12:H15)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="J16" s="3" t="s">
+    <row r="17" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="J17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K16" s="4">
-        <f>1-G8/C7</f>
+      <c r="K17" s="4">
+        <f>1-(SUM(G4:G6))/C7</f>
+        <v>0.55168048309139261</v>
+      </c>
+    </row>
+    <row r="19" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F19" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+    </row>
+    <row r="20" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F20" t="s">
         <v>0</v>
       </c>
+      <c r="G20" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F21" t="s">
+        <v>3</v>
+      </c>
+      <c r="G21" s="2">
+        <f>G4/$K$4</f>
+        <v>0.19827331504955736</v>
+      </c>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F22" t="s">
+        <v>4</v>
+      </c>
+      <c r="G22" s="2">
+        <f>G5/$K$4</f>
+        <v>0.4240792845377544</v>
+      </c>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F23" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="2">
+        <f>G6/$K$4</f>
+        <v>0.37764740041268813</v>
+      </c>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="F19:H19"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="J10:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -824,28 +890,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B17609A2-A501-41D4-9B3C-7FBDBE908257}">
-  <dimension ref="B2:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:L26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -865,7 +931,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -884,8 +950,15 @@
       <c r="H4" s="1">
         <v>0.63667657005</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="1">
+        <f>SUM(G4:G6)</f>
+        <v>4268.4282687687682</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -905,7 +978,7 @@
         <v>2.2010703599362498</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -925,213 +998,299 @@
         <v>8.5582202437500001</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="C7" s="1">
         <v>6384.5624624624634</v>
       </c>
       <c r="D7" s="1">
         <v>17.045680437750001</v>
       </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
       <c r="G7" s="1">
-        <v>4268.4282687687682</v>
+        <f>C7-SUM(G4:G6)</f>
+        <v>2116.1341936936951</v>
       </c>
       <c r="H7" s="1">
-        <v>11.395967173736249</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
+        <f>D7-SUM(H4:H6)</f>
+        <v>5.6497132640137515</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="G8" s="5">
+        <f>SUM(G4:G7)</f>
+        <v>6384.5624624624634</v>
+      </c>
+      <c r="H8" s="5">
+        <f>SUM(H4:H7)</f>
+        <v>17.045680437750001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="F9" s="5" t="s">
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="F10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="J9" s="5" t="s">
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="J10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
         <v>0</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>8</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F11" t="s">
         <v>0</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G11" t="s">
         <v>8</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H11" t="s">
         <v>9</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J11" t="s">
         <v>0</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K11" t="s">
         <v>8</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C12" s="2">
         <f>C4/$C$7</f>
         <v>0.1941965588636215</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D12" s="2">
         <f>D4/$D$7</f>
         <v>0.19419655886362153</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F12" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="2">
-        <f>G4/$G$7</f>
-        <v>5.5868585820194237E-2</v>
-      </c>
-      <c r="H11" s="2">
-        <f>H4/$H$7</f>
-        <v>5.5868585820194237E-2</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="G12" s="2">
+        <f>G4/$G$8</f>
+        <v>3.7351197118537557E-2</v>
+      </c>
+      <c r="H12" s="2">
+        <f>H4/$H$8</f>
+        <v>3.7351197118537564E-2</v>
+      </c>
+      <c r="J12" t="s">
         <v>3</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K12" s="2">
         <f>G4/$C$7</f>
         <v>3.7351197118537557E-2</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L12" s="2">
         <f>H4/$D$7</f>
         <v>3.7351197118537564E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="2">
-        <f t="shared" ref="C12:C13" si="0">C5/$C$7</f>
+      <c r="C13" s="2">
+        <f>C5/$C$7</f>
         <v>0.30372784051696017</v>
       </c>
-      <c r="D12" s="2">
-        <f t="shared" ref="D12:D13" si="1">D5/$D$7</f>
+      <c r="D13" s="2">
+        <f>D5/$D$7</f>
         <v>0.30372784051696017</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="2">
-        <f t="shared" ref="G12:G13" si="2">G5/$G$7</f>
-        <v>0.1931446735832088</v>
-      </c>
-      <c r="H12" s="2">
-        <f t="shared" ref="H12:H13" si="3">H5/$H$7</f>
-        <v>0.19314467358320875</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="G13" s="2">
+        <f t="shared" ref="G13:G14" si="0">G5/$G$8</f>
+        <v>0.12912774987038225</v>
+      </c>
+      <c r="H13" s="2">
+        <f t="shared" ref="H13:H14" si="1">H5/$H$8</f>
+        <v>0.12912774987038225</v>
+      </c>
+      <c r="J13" t="s">
         <v>4</v>
       </c>
-      <c r="K12" s="2">
-        <f t="shared" ref="K12" si="4">G5/$C$7</f>
+      <c r="K13" s="2">
+        <f>G5/$C$7</f>
         <v>0.12912774987038225</v>
       </c>
-      <c r="L12" s="2">
-        <f t="shared" ref="L12:L13" si="5">H5/$D$7</f>
+      <c r="L13" s="2">
+        <f>H5/$D$7</f>
         <v>0.12912774987038225</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C14" s="2">
+        <f>C6/$C$7</f>
+        <v>0.50207560061941825</v>
+      </c>
+      <c r="D14" s="2">
+        <f>D6/$D$7</f>
+        <v>0.50207560061941825</v>
+      </c>
+      <c r="F14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="2">
         <f t="shared" si="0"/>
-        <v>0.50207560061941825</v>
-      </c>
-      <c r="D13" s="2">
+        <v>0.50207560061941814</v>
+      </c>
+      <c r="H14" s="2">
         <f t="shared" si="1"/>
         <v>0.50207560061941825</v>
       </c>
-      <c r="F13" t="s">
+      <c r="J14" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="2">
-        <f t="shared" si="2"/>
-        <v>0.75098674059659698</v>
-      </c>
-      <c r="H13" s="2">
-        <f t="shared" si="3"/>
-        <v>0.75098674059659709</v>
-      </c>
-      <c r="J13" t="s">
-        <v>7</v>
-      </c>
-      <c r="K13" s="2">
+      <c r="K14" s="2">
         <f>G6/$C$7</f>
         <v>0.50207560061941814</v>
       </c>
-      <c r="L13" s="2">
-        <f t="shared" si="5"/>
+      <c r="L14" s="2">
+        <f>H6/$D$7</f>
         <v>0.50207560061941825</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C14" s="2">
-        <f>SUM(C11:C13)</f>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C15" s="2">
+        <f>SUM(C12:C14)</f>
         <v>0.99999999999999989</v>
       </c>
-      <c r="D14" s="2">
-        <f>SUM(D11:D13)</f>
+      <c r="D15" s="2">
+        <f>SUM(D12:D14)</f>
         <v>1</v>
       </c>
-      <c r="G14" s="2">
-        <f>SUM(G11:G13)</f>
+      <c r="F15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="4">
+        <f>G7/$G$8</f>
+        <v>0.33144545239166207</v>
+      </c>
+      <c r="H15" s="4">
+        <f>H7/$H$8</f>
+        <v>0.33144545239166195</v>
+      </c>
+      <c r="K15" s="2">
+        <f>SUM(K12:K14)</f>
+        <v>0.66855454760833788</v>
+      </c>
+      <c r="L15" s="2">
+        <f>SUM(L12:L14)</f>
+        <v>0.6685545476083381</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="G16" s="6">
+        <f>SUM(G12:G15)</f>
         <v>1</v>
       </c>
-      <c r="H14" s="2">
-        <f>SUM(H11:H13)</f>
+      <c r="H16" s="6">
+        <f>SUM(H12:H15)</f>
         <v>1</v>
       </c>
-      <c r="K14" s="2">
-        <f>SUM(K11:K13)</f>
+    </row>
+    <row r="17" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="J17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K17" s="4">
+        <f>1-G7/C7</f>
         <v>0.66855454760833788</v>
       </c>
-      <c r="L14" s="2">
-        <f>SUM(L11:L13)</f>
-        <v>0.6685545476083381</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="J16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K16" s="4">
-        <f>1-G7/C7</f>
-        <v>0.33144545239166201</v>
-      </c>
+    </row>
+    <row r="20" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F20" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+    </row>
+    <row r="21" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F21" t="s">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F22" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="2">
+        <f>G4/$K$4</f>
+        <v>5.5868585820194237E-2</v>
+      </c>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G23" s="2">
+        <f>G5/$K$4</f>
+        <v>0.1931446735832088</v>
+      </c>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F24" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="2">
+        <f>G6/$K$4</f>
+        <v>0.75098674059659698</v>
+      </c>
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="F25" s="3"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" spans="6:11" x14ac:dyDescent="0.35">
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="F20:H20"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="J10:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>